<commit_message>
Stop offering fellowships where they can't be held; prepare v1.6.0
Fellowships
- A fellowship that doesn't say where it can be held was treated as
  open anywhere, so US-only fellowships were offered in India. Not
  stated now means worth checking; only host_countries ["any"] means
  anywhere.
- Host countries filled in for the verified entries whose rules make
  them clear (Damon Runyon, Jane Coffin Childs, LSRF, Helen Hay Whitney,
  NIH F32, ADA, BWF CASI, Grass, EMBL; HFSP, Branco Weiss, Breakthrough
  T1D and Schmidt anywhere; Novo Nordisk, SNSF and Tata abroad only).
- The importer keeps "any"; the template explains blank vs any.

Release
- Version 1.6.0, with release notes.
- The build can be run by hand with a version to release. A single
  release job attaches both apps, to rahulnccs/galley when
  PUBLIC_REPO_TOKEN is set and to this repository otherwise, so a
  release never goes out without its apps.
</commit_message>
<xml_diff>
--- a/templates/fellowship-database-template.xlsx
+++ b/templates/fellowship-database-template.xlsx
@@ -322,7 +322,7 @@
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>Where the fellowship must be held. Blank = anywhere.</t>
+        <t>Where it must be held: two-letter codes, e.g. US, or any if it can be held anywhere. Blank means not stated, shown to users as worth checking.</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
@@ -879,7 +879,7 @@
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Countries: two-letter codes separated by commas, e.g. IN, DE, GB, US. Blank means no restriction.</t>
+          <t>Countries: two-letter codes separated by commas, e.g. IN, DE, GB, US. For host_countries, write any if it can be held anywhere; blank means not stated, which Galley shows as worth checking. For the other country columns, blank means no restriction.</t>
         </is>
       </c>
     </row>
@@ -942,6 +942,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>

</xml_diff>